<commit_message>
AutomaTivio: relatório fiel ao publicado de agosto/2026, taxas dos ALT e PDF selecionável
- Folha A4 redesenhada sobre os PDFs publicados (Institucional 30 e ALT 180):
  cabeçalho preto com logo horizontal e o T, painel do topo, barras e rating
  no desenho do original, histórico desde o início, comentário, mercado de
  crédito, características em duas colunas, disclaimer e rodapé.
- Treemap da alocação real com legenda.
- Taxas e performance dos ALT 180, 90 e Light pelo relatório publicado
  (configs/fundos.yml vence a taxas_global.xlsx).
- PDF: conferência pós-geração (páginas, A4, texto selecionável) e comando
  avulso `python -m exporters.pdf`, no padrão da skill html-to-pdf. O botão
  "PDF (baixar)" da página ganha camada de texto selecionável.
- Saída de agosto/2026 regenerada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -835,7 +835,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+50'], ['Benchmark', 'CDI'], ['Taxa de Performance', 'Não há'], ['Taxa global', '0,65% a.a.'], ['PL (desde o início)', 'R$ 26,8 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+50'], ['Benchmark', 'CDI'], ['Taxa de Performance', '15% do retorno que exceder CDI+0,65%'], ['Taxa global', '1,15% a.a.'], ['PL (desde o início)', 'R$ 26,8 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidores qualificados, Multi Family e Family Offices'], ['Resgate', 'D+180'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder o CDI'], ['Taxa global', '1,15% a.a.'], ['PL Médio (12M)', 'R$ 94,5 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidores qualificados, Multi Family e Family Offices'], ['Resgate', 'D+180'], ['Benchmark', 'CDI'], ['Taxa de Performance', '20% do que exceder do CDI'], ['Taxa global', '1,15% a.a.'], ['PL Médio (12M)', 'R$ 94,5 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+90'], ['Benchmark', 'CDI'], ['Taxa de Performance', '10% do que exceder o CDI'], ['Taxa global', '2,43% a.a.'], ['PL Médio (12M)', 'R$ 15,7 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
+          <t>[['Público Alvo', 'Investidor qualificado'], ['Resgate', 'D+90'], ['Benchmark', 'CDI'], ['Taxa de Performance', '10% do que exceder do CDI'], ['Taxa global', '1,25% a.a.'], ['PL Médio (12M)', 'R$ 15,7 mi'], ['Aplicação Mínima', 'R$ 1.000,00']]</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Taxa global: 2,43% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
+          <t>Taxa global: 1,25% a.a. Taxa de performance: 10% do que exceder do CDI. Resgate: D+90.</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Taxa global: 0,65% a.a. Taxa de performance: não há.</t>
+          <t>Taxa global: 1,15% a.a. Taxa de performance: 15% do retorno que exceder CDI+0,65%.</t>
         </is>
       </c>
     </row>
@@ -12550,7 +12550,7 @@
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -12831,7 +12831,11 @@
           <t>1,15% a.a.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>20% do que exceder do CDI</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>sim</t>
@@ -12856,10 +12860,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2,43% a.a.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>1,25% a.a.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>10% do que exceder do CDI</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>sim</t>
@@ -12884,12 +12892,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,65% a.a.</t>
+          <t>1,15% a.a.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Não há</t>
+          <t>15% do retorno que exceder CDI+0,65%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -13229,11 +13237,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="58" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -13359,287 +13367,66 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>relatorio/banks</t>
+          <t>relatorio/credito_privado</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tivio Banks - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>relatorio/institucional</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tivio Institucional - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é agosto</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>relatorio/inst15</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15 - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
+          <t>sem dados — rentabilidade e PL mantidos</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>relatorio/inst30</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>relatorio/infraplus</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>relatorio/bvp</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Tivio BVP - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>relatorio/rfcp</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Tivio RF CP - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>relatorio/alt180</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180 - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>relatorio/alt90</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90 - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>relatorio/altlight</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>relatorio/infrapluscdi</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>relatorio/esplanada</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>relatorio/legacy</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>fonte Versos não carregou (CDN inacessível?) — o PDF sai com a fonte de fallback e a métrica do texto muda</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>relatorio/credito_privado</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>bvp</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>tivio-email-fundos-credito.html</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>alt180</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é agosto</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>tivio-post-investment-solutions.html</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>topgestormacro</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -13693,7 +13480,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>726075</v>
+        <v>704633</v>
       </c>
     </row>
     <row r="3">
@@ -13708,7 +13495,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>47631</v>
+        <v>47632</v>
       </c>
     </row>
     <row r="4">
@@ -13723,7 +13510,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>735702</v>
+        <v>710959</v>
       </c>
     </row>
     <row r="5">
@@ -13738,7 +13525,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>47824</v>
+        <v>47827</v>
       </c>
     </row>
     <row r="6">
@@ -13753,7 +13540,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>738232</v>
+        <v>714908</v>
       </c>
     </row>
     <row r="7">
@@ -13768,7 +13555,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>47846</v>
+        <v>47847</v>
       </c>
     </row>
     <row r="8">
@@ -13783,7 +13570,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>735788</v>
+        <v>713283</v>
       </c>
     </row>
     <row r="9">
@@ -13798,7 +13585,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>47696</v>
+        <v>47693</v>
       </c>
     </row>
     <row r="10">
@@ -13813,7 +13600,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>722777</v>
+        <v>701041</v>
       </c>
     </row>
     <row r="11">
@@ -13828,7 +13615,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46723</v>
+        <v>46725</v>
       </c>
     </row>
     <row r="12">
@@ -13843,7 +13630,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>725091</v>
+        <v>695670</v>
       </c>
     </row>
     <row r="13">
@@ -13858,7 +13645,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>47653</v>
+        <v>47654</v>
       </c>
     </row>
     <row r="14">
@@ -13873,7 +13660,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>725922</v>
+        <v>704831</v>
       </c>
     </row>
     <row r="15">
@@ -13888,7 +13675,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>47692</v>
+        <v>47696</v>
       </c>
     </row>
     <row r="16">
@@ -13903,7 +13690,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>654116</v>
+        <v>625363</v>
       </c>
     </row>
     <row r="17">
@@ -13918,7 +13705,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>43430</v>
+        <v>43631</v>
       </c>
     </row>
     <row r="18">
@@ -13933,7 +13720,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>646161</v>
+        <v>624108</v>
       </c>
     </row>
     <row r="19">
@@ -13948,7 +13735,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>43362</v>
+        <v>43543</v>
       </c>
     </row>
     <row r="20">
@@ -13963,7 +13750,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>658504</v>
+        <v>625103</v>
       </c>
     </row>
     <row r="21">
@@ -13978,7 +13765,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42241</v>
+        <v>42431</v>
       </c>
     </row>
     <row r="22">
@@ -13993,7 +13780,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>728823</v>
+        <v>704469</v>
       </c>
     </row>
     <row r="23">
@@ -14008,7 +13795,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>47120</v>
+        <v>47123</v>
       </c>
     </row>
     <row r="24">
@@ -14023,7 +13810,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>722104</v>
+        <v>706708</v>
       </c>
     </row>
     <row r="25">
@@ -14038,7 +13825,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>46716</v>
+        <v>46715</v>
       </c>
     </row>
     <row r="26">
@@ -14053,7 +13840,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>726072</v>
+        <v>712840</v>
       </c>
     </row>
     <row r="27">
@@ -14068,7 +13855,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>47687</v>
+        <v>47688</v>
       </c>
     </row>
     <row r="28">
@@ -14083,7 +13870,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3084971</v>
+        <v>3212506</v>
       </c>
     </row>
     <row r="29">
@@ -14098,7 +13885,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1018985</v>
+        <v>1055001</v>
       </c>
     </row>
     <row r="30">
@@ -14113,7 +13900,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>87214</v>
+        <v>88026</v>
       </c>
     </row>
     <row r="31">
@@ -14128,7 +13915,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>130928</v>
+        <v>131775</v>
       </c>
     </row>
     <row r="32">
@@ -14143,7 +13930,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>49750</v>
+        <v>50202</v>
       </c>
     </row>
     <row r="33">
@@ -14158,7 +13945,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>113302</v>
+        <v>114702</v>
       </c>
     </row>
     <row r="34">
@@ -14173,7 +13960,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>126116</v>
+        <v>127504</v>
       </c>
     </row>
     <row r="35">
@@ -14188,7 +13975,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>103643</v>
+        <v>104943</v>
       </c>
     </row>
     <row r="36">
@@ -14203,7 +13990,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>121950</v>
+        <v>122525</v>
       </c>
     </row>
     <row r="37">
@@ -14218,7 +14005,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>66082</v>
+        <v>66613</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AutomaTivio: e-mail com logos horizontais, versão Quadrado e seleção; post IS espaçado
- E-mail: logos sempre na versão horizontal, gerados de assets/logos
  (renderers/logos.py) — branca no modo escuro, preta no claro.
- E-mail: nova versão "Quadrado" (700x700, PNG 2100x2100) com a
  rentabilidade em destaque (12M, Ano, Mês e % do benchmark) e o botão.
- E-mail: caixa "Incluir" por fundo; desmarcado fica fora do "Baixar
  tudo" e do e-mail completo.
- Post Investment Solutions: blocos distribuídos na altura da ficha e
  taxa de performance longa quebrando linha em vez de cortar.
- Gráficos: sem aviso de ECharts quando não há contêiner para ele.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -13480,7 +13480,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>704633</v>
+        <v>832184</v>
       </c>
     </row>
     <row r="3">
@@ -13495,7 +13495,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>47632</v>
+        <v>47637</v>
       </c>
     </row>
     <row r="4">
@@ -13510,7 +13510,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>710959</v>
+        <v>838500</v>
       </c>
     </row>
     <row r="5">
@@ -13525,7 +13525,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>47827</v>
+        <v>47824</v>
       </c>
     </row>
     <row r="6">
@@ -13540,7 +13540,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>714908</v>
+        <v>842446</v>
       </c>
     </row>
     <row r="7">
@@ -13555,7 +13555,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>47847</v>
+        <v>47848</v>
       </c>
     </row>
     <row r="8">
@@ -13570,7 +13570,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>713283</v>
+        <v>840983</v>
       </c>
     </row>
     <row r="9">
@@ -13585,7 +13585,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>47693</v>
+        <v>47696</v>
       </c>
     </row>
     <row r="10">
@@ -13600,7 +13600,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>701041</v>
+        <v>791785</v>
       </c>
     </row>
     <row r="11">
@@ -13615,7 +13615,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46725</v>
+        <v>46722</v>
       </c>
     </row>
     <row r="12">
@@ -13630,7 +13630,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>695670</v>
+        <v>823202</v>
       </c>
     </row>
     <row r="13">
@@ -13645,7 +13645,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>47654</v>
+        <v>47651</v>
       </c>
     </row>
     <row r="14">
@@ -13660,7 +13660,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>704831</v>
+        <v>832443</v>
       </c>
     </row>
     <row r="15">
@@ -13675,7 +13675,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>47696</v>
+        <v>47697</v>
       </c>
     </row>
     <row r="16">
@@ -13735,7 +13735,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>43543</v>
+        <v>43545</v>
       </c>
     </row>
     <row r="20">
@@ -13765,7 +13765,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42431</v>
+        <v>42429</v>
       </c>
     </row>
     <row r="22">
@@ -13780,7 +13780,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>704469</v>
+        <v>832111</v>
       </c>
     </row>
     <row r="23">
@@ -13795,7 +13795,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>47123</v>
+        <v>47118</v>
       </c>
     </row>
     <row r="24">
@@ -13810,7 +13810,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>706708</v>
+        <v>797583</v>
       </c>
     </row>
     <row r="25">
@@ -13825,7 +13825,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>46715</v>
+        <v>46717</v>
       </c>
     </row>
     <row r="26">
@@ -13840,7 +13840,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>712840</v>
+        <v>840434</v>
       </c>
     </row>
     <row r="27">
@@ -13855,7 +13855,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>47688</v>
+        <v>47685</v>
       </c>
     </row>
     <row r="28">
@@ -13870,7 +13870,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3212506</v>
+        <v>3218147</v>
       </c>
     </row>
     <row r="29">
@@ -13885,7 +13885,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1055001</v>
+        <v>1060312</v>
       </c>
     </row>
     <row r="30">
@@ -13915,7 +13915,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>131775</v>
+        <v>176798</v>
       </c>
     </row>
     <row r="32">
@@ -13975,7 +13975,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>104943</v>
+        <v>105529</v>
       </c>
     </row>
     <row r="36">

</xml_diff>

<commit_message>
AutomaTivio: PPTX fiel à folha com texto editável; logos em curvas; T e Central
- PPTX: novo exporters/pptx_fiel.py (abordagem "Image to PPTX" da skill
  ppt-master): fundo = folha renderizada sem texto; por cima, cada bloco
  de texto como caixa nativa editável, na posição e estilo medidos no
  Chromium. O "nativo" antigo (outro layout) fica só como reserva.
- Logos Legacy e Esplanada: o texto digitado (<text> em Versos) virou
  curvas, com o espaçamento do Illustrator.
- Cabeçalho: caixa do T volta ao cinza escuro do publicado (uma regra
  antiga a deixava transparente) e o T no tamanho e posição do modelo.
- Central: sai o gerador antigo tivio-relatorio-gestao-credito-privado.html
  (fonte guardada em templates/referencia/, de onde saiu o pagina.css).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -424,10 +424,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
@@ -4568,2181 +4568,210 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>mercado</t>
+          <t>s1</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>MARKET</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>[['Total', '446.217', '100,0%', '1,14%', '1,17%', '-0,03%', '2,86', True], ['Energia elétrica', '102.982', '23,11%', '0,75%', '0,76%', '-0,02%', '2,78', False], ['Assistência médica', '45.853', '10,29%', '1,45%', '1,48%', '-0,04%', '3,40', False], ['Locação de veículos', '43.937', '9,86%', '1,72%', '1,71%', '0,02%', '2,51', False], ['Saneamento', '40.735', '9,14%', '1,43%', '1,44%', '-0,01%', '2,87', False], ['Petróleo e gás', '33.732', '7,57%', '0,91%', '0,95%', '-0,04%', '3,01', False], ['Transporte e logística', '27.250', '6,11%', '1,41%', '1,54%', '-0,12%', '2,78', False], ['Comércio atacadista e varejista', '24.639', '5,53%', '1,33%', '1,39%', '-0,06%', '2,65', False], ['Financeiro', '23.379', '5,25%', '0,52%', '0,54%', '-0,02%', '2,38', False], ['Indústria e comércio', '20.251', '4,54%', '1,15%', '1,20%', '-0,04%', '2,82', False], ['TI e telecomunicações', '17.577', '3,94%', '1,11%', '1,12%', '-0,01%', '2,46', False], ['Bioenergia', '11.334', '2,54%', '1,74%', '1,80%', '-0,06%', '3,08', False], ['Metalurgia e siderurgia', '9.560', '2,15%', '1,25%', '1,15%', '0,10%', '3,10', False], ['Educação', '7.933', '1,78%', '1,02%', '1,06%', '-0,04%', '2,39', False], ['Outros serviços', '7.003', '1,57%', '1,10%', '1,12%', '-0,02%', '2,89', False], ['Empreendimentos e participações', '6.693', '1,50%', '1,23%', '1,24%', '-0,01%', '3,44', False], ['Serviços imobiliários', '6.353', '1,43%', '0,64%', '0,65%', '-0,01%', '3,62', False], ['Papel e Celulose', '5.247', '1,18%', '0,58%', '0,60%', '-0,03%', '4,73', False], ['Materiais de construção e agregados', '4.144', '0,93%', '1,04%', '1,04%', '0,00%', '3,64', False], ['Química e petroquímica', '2.554', '0,57%', '1,11%', '1,14%', '-0,03%', '3,75', False], ['Alimentos e bebidas', '1.727', '0,39%', '1,25%', '1,28%', '-0,03%', '1,37', False], ['Têxtil e calçados', '1.528', '0,34%', '1,25%', '1,25%', '0,00%', '2,90', False], ['Mineração', '1.072', '0,24%', '0,83%', '0,86%', '-0,03%', '2,51', False], ['Construção civil', '166', '0,04%', '1,66%', '1,82%', '-0,16%', '0,68', False]]</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>[['Setor', 'Volume (R$ MM)', '%', 'Spread Atual', 'Spread mês anterior', 'Variação', 'Duration', False], ['Total', '(a linha Total vem primeiro)', '', '', '', '', '', True]]</t>
+          <t>Agosto 2026</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>s2</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>pl</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>R$ 1.698.520.740,05</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>R$ 1.793.381.077,96</t>
+          <t>Agosto 2026</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>s8</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>plm</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>R$ 1.397.203.402,03</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>R$ 1.449.683.179,97</t>
+          <t>Agosto 2026</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>e1</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>perfrows</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>{'pct': ['101%', '100%', '100%']}</t>
+          <t>Julho 2026</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>{'fundo': ['1,10%', '9,36%', '14,63%', '29,82%', '45,41%', '444,67%'], 'bench': ['1,09%', '9,33%', '14,57%', '29,49%', '44,17%', '408,92%'], 'pct': ['100,59%', '100,31%', '100,43%', '101,12%', '102,80%', '108,74%'], 'alfa': ['0,01%', '0,03%', '0,06%', '0,33%', '1,24%', '35,75%']}</t>
+          <t>Agosto 2026</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>emissores</t>
+          <t>title</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>[['ITAÚ UNIBANCO', '3,42%', 100], ['BRADESCO', '3,18%', 93], ['SANTANDER', '2,86%', 84], ['BANCO DO BRASIL', '2,54%', 74], ['BTG PACTUAL', '2,21%', 65]]</t>
+          <t>Relatório de Gestão · Incentivado CDI 30</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>[['BV', '6,36%', 100], ['XP', '6,04%', 95], ['BTG', '5,97%', 94], ['ABC', '5,92%', 93], ['NUBANK', '5,57%', 88]]</t>
+          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>setores</t>
+          <t>desc</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>[['Financeiro', '76,5%'], ['Caixa', '23,5%']]</t>
+          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>[['Financeiro', '75,7%'], ['Caixa', '24,2%']]</t>
+          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>rating</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>[['AAA', '46,2%', 100], ['AA+', '24,8%', 54], ['AA', '14,1%', 31], ['AA-', '9,4%', 20], ['A+', '3,9%', 8], ['A', '1,6%', 3]]</t>
+          <t>cards de relatório</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>[['AAA', '50,8%', 100], ['AA+', '16,3%', 32], ['AA', '2,0%', 4], ['A+', '1,9%', 4], ['A', '3,0%', 6]]</t>
+          <t>2 registrados para Agosto 2026</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>0,26%</t>
-        </is>
-      </c>
+          <t>data automática</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
-        <is>
-          <t>0,25%</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>banks</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>1,12</t>
-        </is>
-      </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>1,05</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>banks</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>hist12</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t>{'b': 'CDI', 'l': ['2025-08', '2025-09', '2025-10', '2025-11', '2025-12', '2026-01', '2026-02', '2026-03', '2026-04', '2026-05', '2026-06', '2026-07', '2026-08'], 'f': [0.0, 1.23, 2.53, 3.62, 4.88, 6.11, 7.18, 8.48, 9.64, 10.82, 12.07, 13.45, 14.7], 'c': [0.0, 1.22, 2.51, 3.59, 4.85, 6.07, 7.13, 8.43, 9.61, 10.79, 12.03, 13.39, 14.63]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>banks</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>histEnd</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>[12.0, 12.0, 'CDI']</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>[14.7, 14.63, 'CDI']</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>banks</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>comentario</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>['No mês, o mercado de crédito privado high grade manteve o movimento de fechamento gradual de spreads, com fluxo comprador consistente no secundário e oferta primária ainda concentrada em emissores de primeira linha.', 'A liquidez permaneceu saudável ao longo da curva, com boa demanda por papéis bancários e por debêntures de empresas de energia, saneamento e infraestrutura, setores de maior peso na carteira.', 'Do ponto de vista da gestão, seguimos priorizando emissores de baixo risco de crédito e o controle da duration, mantendo carrego atrativo sobre o CDI sem elevar de forma relevante a volatilidade da cota.', 'O BANKS apresentou rentabilidade de &lt;b&gt;1,01%&lt;/b&gt; no mês (&lt;b&gt;101% do CDI&lt;/b&gt;), acumulando &lt;b&gt;8,17%&lt;/b&gt; no ano. Os principais atribuidores de resultado foram as debêntures corporativas e a parcela bancária da carteira.']</t>
-        </is>
-      </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>['O Fundo Tivio Banks obteve retorno de 1,10% (101% do CDI) no mês e acumula 9,36% (100% do CDI) em 2026. A alocação em crédito era de 75%, integralmente concentrada em emissores do setor bancário. O carrego da carteira encontra-se em CDI +0,25%, com duration média de 1,05 ano.', 'Em agosto, o mercado de crédito foi marcado por um ambiente de menor liquidez nas negociações do mercado secundário e por uma leve reabertura dos spreads de crédito. Após meses consecutivos de compressão dos prêmios de risco, observou-se um movimento mais cauteloso por parte dos investidores, com os spreads médios dos títulos corporativos indexados ao CDI avançando aproximadamente 0,03%, passando de CDI + 1,19% para CDI + 1,22% ao ano. Apesar desse ajuste, os níveis de prêmio permaneceram próximos das mínimas históricas observadas ao longo do ciclo recente.', 'No mercado secundário, a redução do volume negociado contribuiu para uma formação de preços mais seletiva, especialmente em ativos corporativos com menor liquidez. Ainda assim, o comportamento dos investidores permaneceu construtivo, sustentado por um ambiente técnico favorável e pela continuidade da elevada demanda por ativos de crédito.', 'Já no mercado primário, as emissões bancárias seguiram registrando forte demanda por parte dos investidores. As ofertas de Letras Financeiras Seniores distribuídas ao longo do mês apresentaram níveis elevados de subscrição, com demanda que, em diversos casos, superou três vezes o volume ofertado. Esse forte apetite permitiu que as operações fossem precificadas com taxas inferiores aos limites inicialmente indicados pelos emissores, evidenciando a elevada disponibilidade de recursos para alocação na indústria de crédito.', 'Em relação aos fluxos, os fundos com alocação mínima de 15% em crédito e ao menos 1% em debêntures apresentaram captação líquida próxima de R$ 8 bilhões em agosto, resultado significativamente superior ao observado no mês anterior. O volume reforça a percepção de que os investidores seguem direcionando recursos para estratégias de crédito, impulsionados pelo elevado nível de carrego proporcionado pelos ativos indexados ao CDI e pela busca por alternativas de investimento com perfil de risco-retorno atrativo.', 'Nesse contexto, a combinação entre fluxos positivos para a indústria, vencimentos e amortizações recorrentes das carteiras, além da limitada oferta de novos ativos corporativos, continuou sustentando a demanda por crédito privado. Ainda que agosto tenha apresentado uma leve reabertura dos spreads médios de mercado, a dinâmica técnica permanece favorável e os prêmios seguem negociando em patamares historicamente reduzidos.', 'Por fim, sob a ótica da gestão, seguimos acompanhando de forma criteriosa a evolução dos fundamentos dos emissores presentes nas carteiras, com atenção especial aos indicadores operacionais, à geração de caixa e à manutenção de estruturas de capital adequadas. Em um ambiente em que os spreads permanecem comprimidos em termos históricos, mantemos disciplina na alocação dos recursos, priorizando operações que apresentem adequada relação entre risco e retorno e preservando flexibilidade para captura de oportunidades que possam surgir em eventuais períodos de maior volatilidade do mercado.']</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>pl</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>R$ 1.983.487.947,49</t>
-        </is>
-      </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>R$ 1.815.644.128,24</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>plm</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>R$ 2.522.009.705,73</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>R$ 2.491.331.200,61</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>perfrows</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>{'pct': ['104%', '100%', '100%']}</t>
-        </is>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>{'fundo': ['1,09%', '9,31%', '14,58%', '29,93%', '47,60%', '825,45%'], 'bench': ['1,09%', '9,33%', '14,57%', '29,49%', '44,17%', '753,88%'], 'pct': ['100%', '100%', '100%', '102%', '108%', '109%'], 'alfa': ['−0,01%', '−0,02%', '0,01%', '0,44%', '3,43%', '71,57%']}</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>emissores</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>[['AEGEA', '2,64%', 100], ['TUPY', '2,31%', 88], ['VALE', '2,05%', 78], ['PETROBRAS', '1,86%', 70], ['RANDON', '1,52%', 58]]</t>
-        </is>
-      </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>[['BTG', '3,45%', 100], ['BB', '3,44%', 100], ['SANTANDER', '3,06%', 89], ['SAFRA', '3,02%', 88], ['BRADESCO', '2,89%', 84]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>setores</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>[['Financeiro', '52%'], ['Energia Elétrica', '4%'], ['Transporte e Logística', '2%'], ['Saneamento', '2%'], ['Caixa', '31%']]</t>
-        </is>
-      </c>
-      <c r="E170" t="inlineStr">
-        <is>
-          <t>[['Financeiro', '44,6%'], ['Energia Elétrica', '4,5%'], ['FIDC', '2,1%'], ['Transporte e Logística', '2,1%'], ['Saneamento', '2,0%'], ['Caixa', '38,7%']]</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>[['AAA', '46,2%', 100], ['AA+', '24,8%', 54], ['AA', '14,1%', 31], ['AA-', '9,4%', 20], ['A+', '3,9%', 8], ['A', '1,6%', 3]]</t>
-        </is>
-      </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>[['AAA', '39,6%', 100], ['AA+', '10,5%', 27], ['AA', '2,4%', 6], ['AA-', '2,7%', 7], ['A+', '1,2%', 3], ['A', '3,3%', 8]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>0,44%</t>
-        </is>
-      </c>
-      <c r="E172" t="inlineStr">
-        <is>
-          <t>0,39%</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>1,20</t>
-        </is>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>1,28</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>hist12</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>{'b': 'CDI', 'l': ['2025-08', '2025-09', '2025-10', '2025-11', '2025-12', '2026-01', '2026-02', '2026-03', '2026-04', '2026-05', '2026-06', '2026-07', '2026-08'], 'f': [0.0, 1.25, 2.52, 3.59, 4.88, 6.12, 7.13, 8.29, 9.43, 10.74, 11.99, 13.41, 14.64], 'c': [0.0, 1.22, 2.51, 3.59, 4.85, 6.07, 7.13, 8.43, 9.61, 10.79, 12.03, 13.39, 14.63]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>histEnd</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>[12.48, 12.0, 'CDI']</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>[14.64, 14.63, 'CDI']</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>institucional</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>comentario</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>['No mês, o mercado de crédito privado high grade manteve o movimento de fechamento gradual de spreads, com fluxo comprador consistente no secundário e oferta primária ainda concentrada em emissores de primeira linha.', 'A liquidez permaneceu saudável ao longo da curva, com boa demanda por papéis bancários e por debêntures de empresas de energia, saneamento e infraestrutura, setores de maior peso na carteira.', 'Do ponto de vista da gestão, seguimos priorizando emissores de baixo risco de crédito e o controle da duration, mantendo carrego atrativo sobre o CDI sem elevar de forma relevante a volatilidade da cota.', 'O INSTITUCIONAL apresentou rentabilidade de &lt;b&gt;1,27%&lt;/b&gt; no mês (&lt;b&gt;104% do CDI&lt;/b&gt;), acumulando &lt;b&gt;8,13%&lt;/b&gt; no ano. Os principais atribuidores de resultado foram as debêntures corporativas e a parcela bancária da carteira.']</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>['Em agosto, o mercado de crédito foi marcado por um ambiente de menor liquidez nas negociações do mercado secundário e por uma leve reabertura dos spreads de crédito. Após meses consecutivos de compressão dos prêmios de risco, observou-se um movimento mais cauteloso por parte dos investidores, com os spreads médios dos títulos corporativos indexados ao CDI avançando aproximadamente 0,03%, passando de CDI + 1,19% para CDI + 1,22% ao ano. Apesar desse ajuste, os níveis de prêmio permaneceram próximos das mínimas históricas observadas ao longo do ciclo recente.', 'No mercado secundário, a redução do volume negociado contribuiu para uma formação de preços mais seletiva, especialmente em ativos corporativos com menor liquidez. Ainda assim, o comportamento dos investidores permaneceu construtivo, sustentado por um ambiente técnico favorável e pela continuidade da elevada demanda por ativos de crédito.', 'Já no mercado primário, as emissões bancárias seguiram registrando forte demanda por parte dos investidores. As ofertas de Letras Financeiras Seniores distribuídas ao longo do mês apresentaram níveis elevados de subscrição, com demanda que, em diversos casos, superou três vezes o volume ofertado. Esse forte apetite permitiu que as operações fossem precificadas com taxas inferiores aos limites inicialmente indicados pelos emissores, evidenciando a elevada disponibilidade de recursos para alocação na indústria de crédito. Por outro lado, o pipeline de emissões corporativas permaneceu limitado, restringindo a oferta de novos ativos em um momento de demanda ainda aquecida.', 'Em relação aos fluxos, os fundos com alocação mínima de 15% em crédito e ao menos 1% em debêntures apresentaram captação líquida próxima de R$ 8 bilhões em agosto, resultado significativamente superior ao observado no mês anterior. O volume reforça a percepção de que os investidores seguem direcionando recursos para estratégias de crédito, impulsionados pelo elevado nível de carrego proporcionado pelos ativos indexados ao CDI e pela busca por alternativas de investimento com perfil de risco-retorno atrativo.', 'Nesse contexto, a combinação entre fluxos positivos para a indústria, vencimentos e amortizações recorrentes das carteiras, além da limitada oferta de novos ativos corporativos, continuou sustentando a demanda por crédito privado. Ainda que agosto tenha apresentado uma leve reabertura dos spreads médios de mercado, a dinâmica técnica permanece favorável e os prêmios seguem negociando em patamares historicamente reduzidos.', 'Por fim, sob a ótica da gestão, seguimos acompanhando de forma criteriosa a evolução dos fundamentos dos emissores presentes nas carteiras, com atenção especial aos indicadores operacionais, à geração de caixa e à manutenção de estruturas de capital adequadas. Em um ambiente em que os spreads permanecem comprimidos em termos históricos, mantemos disciplina na alocação dos recursos, priorizando operações que apresentem adequada relação entre risco e retorno e preservando flexibilidade para captura de oportunidades que possam surgir em eventuais períodos de maior volatilidade do mercado.', 'Nesse cenário, o Fundo Tivio Institucional apresentou rentabilidade de 1,09% no mês (100% do CDI), acumulando 9,31% (100% do CDI) no ano. Na parcela de corporativos, os maiores atribuidores de resultado foram para Argo e Aegea, enquanto Aegea foi o maior detrator.']</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>adm</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>0,45% a.a.</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>0,50% a.a.</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>perf</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>Não há</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>20% do que exceder 102,5% do CDI</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>pl</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>R$ 161.593.743,98</t>
-        </is>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>R$ 156.046.891,63</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>plm</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>R$ 140.997.685,81</t>
-        </is>
-      </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>R$ 146.843.921,67</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>perfrows</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>{'pct': ['113%', '102%', '102%']}</t>
-        </is>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>{'fundo': ['1,11%', '9,53%', '14,94%', '30,92%', '51,22%', '1.644,37%'], 'bench': ['1,09%', '9,33%', '14,57%', '29,49%', '44,17%', '1.408,13%'], 'pct': ['102%', '102%', '103%', '105%', '116%', '117%'], 'alfa': ['0,02%', '0,20%', '0,36%', '1,43%', '7,05%', '236,24%']}</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>emissores</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>[['TUPY', '3,04%', 100], ['UNIDAS', '2,71%', 89], ['AEGEA', '2,33%', 77], ['HAPVIDA', '2,01%', 66], ['EQUATORIAL', '1,74%', 57]]</t>
-        </is>
-      </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>[['C6', '5,45%', 100], ['ABC', '3,43%', 63], ['XP', '3,28%', 60], ['BTG', '3,28%', 60], ['BRADESCO', '1,76%', 32]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>setores</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>[['Financeiro', '29%'], ['FIDC', '13%'], ['Energia Elétrica', '7%'], ['Saneamento', '5%'], ['Transporte e Logística', '4%'], ['Caixa', '26%']]</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>[['Financeiro', '28,0%'], ['FIDC', '13,0%'], ['Energia Elétrica', '7,1%'], ['Locação de veículos', '3,8%'], ['Saneamento', '3,5%'], ['Caixa', '27,2%']]</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>[['AAA', '46,2%', 100], ['AA+', '24,8%', 54], ['AA', '14,1%', 31], ['AA-', '9,4%', 20], ['A+', '3,9%', 8], ['A', '1,6%', 3]]</t>
-        </is>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>[['AAA', '32,7%', 100], ['AA+', '7,8%', 24], ['AA', '4,1%', 13], ['AA-', '5,7%', 17], ['A+', '4,2%', 13], ['A', '6,2%', 19]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>1,00%</t>
-        </is>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>0,95%</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr">
-        <is>
-          <t>1,97</t>
-        </is>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>1,80</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>anos</t>
-        </is>
-      </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>hist12</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>{'b': 'CDI', 'l': ['2025-08', '2025-09', '2025-10', '2025-11', '2025-12', '2026-01', '2026-02', '2026-03', '2026-04', '2026-05', '2026-06', '2026-07', '2026-08'], 'f': [0.0, 1.29, 2.5, 3.53, 5.0, 6.31, 7.33, 8.3, 9.48, 10.88, 12.2, 13.74, 15.0], 'c': [0.0, 1.22, 2.51, 3.59, 4.85, 6.07, 7.13, 8.43, 9.61, 10.79, 12.03, 13.39, 14.63]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>histEnd</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>[12.24, 12.0, 'CDI']</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>[15.0, 14.63, 'CDI']</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>comentario</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>['No mês, o mercado de crédito privado high grade manteve o movimento de fechamento gradual de spreads, com fluxo comprador consistente no secundário e oferta primária ainda concentrada em emissores de primeira linha.', 'A liquidez permaneceu saudável ao longo da curva, com boa demanda por papéis bancários e por debêntures de empresas de energia, saneamento e infraestrutura, setores de maior peso na carteira.', 'Do ponto de vista da gestão, seguimos priorizando emissores de baixo risco de crédito e o controle da duration, mantendo carrego atrativo sobre o CDI sem elevar de forma relevante a volatilidade da cota.', 'O INSTITUCIONAL 15 apresentou rentabilidade de &lt;b&gt;1,37%&lt;/b&gt; no mês (&lt;b&gt;113% do CDI&lt;/b&gt;), acumulando &lt;b&gt;8,32%&lt;/b&gt; no ano. Os principais atribuidores de resultado foram as debêntures corporativas e a parcela bancária da carteira.']</t>
-        </is>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>['Em agosto, o mercado de crédito foi marcado por um ambiente de menor liquidez nas negociações do mercado secundário e por uma leve reabertura dos spreads de crédito. Após meses consecutivos de compressão dos prêmios de risco, observou-se um movimento mais cauteloso por parte dos investidores, com os spreads médios dos títulos corporativos indexados ao CDI avançando aproximadamente 0,03%, passando de CDI + 1,19% para CDI + 1,22% ao ano. Apesar desse ajuste, os níveis de prêmio permaneceram próximos das mínimas históricas observadas ao longo do ciclo recente.', 'No mercado secundário, a redução do volume negociado contribuiu para uma formação de preços mais seletiva, especialmente em ativos corporativos com menor liquidez. Ainda assim, o comportamento dos investidores permaneceu construtivo, sustentado por um ambiente técnico favorável e pela continuidade da elevada demanda por ativos de crédito.', 'Já no mercado primário, as emissões bancárias seguiram registrando forte demanda por parte dos investidores. As ofertas de Letras Financeiras Seniores distribuídas ao longo do mês apresentaram níveis elevados de subscrição, com demanda que, em diversos casos, superou três vezes o volume ofertado. Esse forte apetite permitiu que as operações fossem precificadas com taxas inferiores aos limites inicialmente indicados pelos emissores, evidenciando a elevada disponibilidade de recursos para alocação na indústria de crédito. Por outro lado, o pipeline de emissões corporativas permaneceu limitado, restringindo a oferta de novos ativos em um momento de demanda ainda aquecida.', 'Em relação aos fluxos, os fundos com alocação mínima de 15% em crédito e ao menos 1% em debêntures apresentaram captação líquida próxima de R$ 8 bilhões em agosto, resultado significativamente superior ao observado no mês anterior. O volume reforça a percepção de que os investidores seguem direcionando recursos para estratégias de crédito, impulsionados pelo elevado nível de carrego proporcionado pelos ativos indexados ao CDI e pela busca por alternativas de investimento com perfil de risco-retorno atrativo.', 'Nesse contexto, a combinação entre fluxos positivos para a indústria, vencimentos e amortizações recorrentes das carteiras, além da limitada oferta de novos ativos corporativos, continuou sustentando a demanda por crédito privado. Ainda que agosto tenha apresentado uma leve reabertura dos spreads médios de mercado, a dinâmica técnica permanece favorável e os prêmios seguem negociando em patamares historicamente reduzidos.', 'Por fim, sob a ótica da gestão, seguimos acompanhando de forma criteriosa a evolução dos fundamentos dos emissores presentes nas carteiras, com atenção especial aos indicadores operacionais, à geração de caixa e à manutenção de estruturas de capital adequadas. Em um ambiente em que os spreads permanecem comprimidos em termos históricos, mantemos disciplina na alocação dos recursos, priorizando operações que apresentem adequada relação entre risco e retorno e preservando flexibilidade para captura de oportunidades que possam surgir em eventuais períodos de maior volatilidade do mercado.', 'Nesse cenário, o Tivio Institucional 15 apresentou rentabilidade de 1,11% no mês (102% do CDI), acumulando 9,53% (102% do CDI) no ano. Na parcela de corporativos, os maiores atribuidores de resultado foram para Tupy e Randon, enquanto Hapvida foi o maior detrator.']</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>adm</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>0,63% a.a.</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>0,625% a.a.</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>perf</t>
-        </is>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>20% do que exceder o CDI</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>20% do que exceder 100% do CDI</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>pl</t>
-        </is>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>R$ 143.232.764,20</t>
-        </is>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>R$ 126.168.780,56</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>plm</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>R$ 155.004.649,74</t>
-        </is>
-      </c>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>R$ 158.893.390,74</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>perfrows</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>{'pct': ['113%', '101%', '101%']}</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>{'fundo': ['1,12%', '9,45%', '14,68%', '−', '−', '25,93%'], 'bench': ['1,09%', '9,33%', '14,57%', '−', '−', '25,71%'], 'pct': ['102%', '101%', '101%', '−', '−', '101%'], 'alfa': ['0,03%', '0,12%', '0,11%', '−', '−', '0,21%']}</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>emissores</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>[['AEGEA', '2,88%', 100], ['EQUATORIAL', '2,55%', 89], ['TUPY', '2,22%', 77], ['SABESP', '1,94%', 67], ['ENGIE', '1,67%', 58]]</t>
-        </is>
-      </c>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>[['C6', '6,00%', 100], ['ABC', '3,78%', 63], ['XP', '3,62%', 60], ['BTG', '3,62%', 60], ['BRADESCO', '1,94%', 32]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>setores</t>
-        </is>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>[['Financeiro', '33%'], ['FIDC', '15%'], ['Energia Elétrica', '8%'], ['Saneamento', '6%'], ['Transporte e Logística', '5%'], ['Caixa', '16%']]</t>
-        </is>
-      </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>[['Financeiro', '30,8%'], ['FIDC', '14,4%'], ['Energia Elétrica', '7,8%'], ['Locação de veículos', '4,2%'], ['Saneamento', '3,8%'], ['Caixa', '19,7%']]</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>[['AAA', '46,2%', 100], ['AA+', '24,8%', 54], ['AA', '14,1%', 31], ['AA-', '9,4%', 20], ['A+', '3,9%', 8], ['A', '1,6%', 3]]</t>
-        </is>
-      </c>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>[['AAA', '36,0%', 100], ['AA+', '8,6%', 24], ['AA', '4,5%', 13], ['AA-', '6,2%', 17], ['A+', '4,7%', 13], ['A', '6,8%', 19]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>1,04%</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E200" t="inlineStr">
-        <is>
-          <t>1,86</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>anos</t>
-        </is>
-      </c>
-      <c r="E201" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>hist12</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>{'b': 'CDI', 'l': ['2025-08', '2025-09', '2025-10', '2025-11', '2025-12', '2026-01', '2026-02', '2026-03', '2026-04', '2026-05', '2026-06', '2026-07', '2026-08'], 'f': [0.0, 1.3, 2.52, 3.56, 4.85, 6.13, 7.14, 8.01, 9.16, 10.62, 11.95, 13.48, 14.75], 'c': [0.0, 1.22, 2.51, 3.59, 4.85, 6.07, 7.13, 8.43, 9.61, 10.79, 12.03, 13.39, 14.63]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C203" t="inlineStr">
-        <is>
-          <t>histEnd</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>[12.12, 12.0, 'CDI']</t>
-        </is>
-      </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>[14.75, 14.63, 'CDI']</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>comentario</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>['No mês, o mercado de crédito privado high grade manteve o movimento de fechamento gradual de spreads, com fluxo comprador consistente no secundário e oferta primária ainda concentrada em emissores de primeira linha.', 'A liquidez permaneceu saudável ao longo da curva, com boa demanda por papéis bancários e por debêntures de empresas de energia, saneamento e infraestrutura, setores de maior peso na carteira.', 'Do ponto de vista da gestão, seguimos priorizando emissores de baixo risco de crédito e o controle da duration, mantendo carrego atrativo sobre o CDI sem elevar de forma relevante a volatilidade da cota.', 'O INSTITUCIONAL 30 apresentou rentabilidade de &lt;b&gt;1,36%&lt;/b&gt; no mês (&lt;b&gt;113% do CDI&lt;/b&gt;), acumulando &lt;b&gt;8,08%&lt;/b&gt; no ano. Os principais atribuidores de resultado foram as debêntures corporativas e a parcela bancária da carteira.']</t>
-        </is>
-      </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>['Em agosto, o mercado de crédito foi marcado por um ambiente de menor liquidez nas negociações do mercado secundário e por uma leve reabertura dos spreads de crédito. Após meses consecutivos de compressão dos prêmios de risco, observou-se um movimento mais cauteloso por parte dos investidores, com os spreads médios dos títulos corporativos indexados ao CDI avançando aproximadamente 0,03%, passando de CDI + 1,19% para CDI + 1,22% ao ano. Apesar desse ajuste, os níveis de prêmio permaneceram próximos das mínimas históricas observadas ao longo do ciclo recente.', 'No mercado secundário, a redução do volume negociado contribuiu para uma formação de preços mais seletiva, especialmente em ativos corporativos com menor liquidez. Ainda assim, o comportamento dos investidores permaneceu construtivo, sustentado por um ambiente técnico favorável e pela continuidade da elevada demanda por ativos de crédito.', 'Já no mercado primário, as emissões bancárias seguiram registrando forte demanda por parte dos investidores. As ofertas de Letras Financeiras Seniores distribuídas ao longo do mês apresentaram níveis elevados de subscrição, com demanda que, em diversos casos, superou três vezes o volume ofertado. Esse forte apetite permitiu que as operações fossem precificadas com taxas inferiores aos limites inicialmente indicados pelos emissores, evidenciando a elevada disponibilidade de recursos para alocação na indústria de crédito. Por outro lado, o pipeline de emissões corporativas permaneceu limitado, restringindo a oferta de novos ativos em um momento de demanda ainda aquecida.', 'Em relação aos fluxos, os fundos com alocação mínima de 15% em crédito e ao menos 1% em debêntures apresentaram captação líquida próxima de R$ 8 bilhões em agosto, resultado significativamente superior ao observado no mês anterior. O volume reforça a percepção de que os investidores seguem direcionando recursos para estratégias de crédito, impulsionados pelo elevado nível de carrego proporcionado pelos ativos indexados ao CDI e pela busca por alternativas de investimento com perfil de risco-retorno atrativo.', 'Nesse contexto, a combinação entre fluxos positivos para a indústria, vencimentos e amortizações recorrentes das carteiras, além da limitada oferta de novos ativos corporativos, continuou sustentando a demanda por crédito privado. Ainda que agosto tenha apresentado uma leve reabertura dos spreads médios de mercado, a dinâmica técnica permanece favorável e os prêmios seguem negociando em patamares historicamente reduzidos.', 'Por fim, sob a ótica da gestão, seguimos acompanhando de forma criteriosa a evolução dos fundamentos dos emissores presentes nas carteiras, com atenção especial aos indicadores operacionais, à geração de caixa e à manutenção de estruturas de capital adequadas. Em um ambiente em que os spreads permanecem comprimidos em termos históricos, mantemos disciplina na alocação dos recursos, priorizando operações que apresentem adequada relação entre risco e retorno e preservando flexibilidade para captura de oportunidades que possam surgir em eventuais períodos de maior volatilidade do mercado.', 'Nesse cenário, o Tivio Institucional 30 apresentou rentabilidade de 1,12% no mês (102% do CDI), acumulando 9,45% (101% do CDI) no ano. Na parcela de corporativos, os maiores atribuidores de resultado foram para Tupy e Randon, enquanto Hapvida foi o maior detrator.']</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>pl</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>R$ 42.983.282,75</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>R$ 42.694.019,75</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>plm</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>R$ 52.049.593,91</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>R$ 49.421.174,50</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>perfrows</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>{'abs': ['1,24%', '7,80%', '12,94%'], 'alfa': ['−0,14%', '−3,14%', '−2,75%']}</t>
-        </is>
-      </c>
-      <c r="E207" t="inlineStr">
-        <is>
-          <t>{'fundo': ['1,26%', '5,98%', '9,91%', '19,03%', '29,49%', '77,41%'], 'bench': ['1,28%', '9,18%', '13,34%', '23,32%', '33,11%', '87,91%'], 'abs': ['1,26%', '5,98%', '9,91%', '19,03%', '29,49%', '77,41%'], 'alfa': ['−0,01%', '−3,20%', '−3,44%', '−4,28%', '−3,62%', '−10,50%']}</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>emissores</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>[['EQUATORIAL', '3,87%', 100], ['CEMIG', '3,42%', 88], ['COPEL', '3,14%', 81], ['SABESP', '3,03%', 78], ['ELETROBRAS', '2,92%', 75]]</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>[['AUREN', '7,68%', 100], ['EQUATORIAL', '7,24%', 94], ['EDF', '5,54%', 72], ['SINOP', '3,99%', 52], ['ELETROBRAS', '3,65%', 48]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>setores</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>[['Energia Elétrica', '55%'], ['Transporte e Logística', '15%'], ['Saneamento', '7%'], ['Petróleo e Gás', '5%'], ['TI e Telecomunicações', '4%'], ['Caixa', '5%']]</t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>[['Energia Elétrica', '55,9%'], ['Transporte e Logística', '15,3%'], ['Saneamento', '7,3%'], ['TI e Telecomunicações', '5,4%'], ['Petróleo e Gás', '4,8%'], ['Caixa', '4,8%']]</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>[['AAA', '32,35%', 100], ['AA+', '17,91%', 55], ['AA', '11,27%', 35], ['AA-', '15,61%', 48], ['A+', '7,15%', 22], ['A', '1,85%', 6]]</t>
-        </is>
-      </c>
-      <c r="E210" t="inlineStr">
-        <is>
-          <t>[['AAA', '35,4%', 100], ['AA+', '26,0%', 74], ['AA', '11,1%', 31], ['AA-', '8,8%', 25], ['A+', '5,1%', 14], ['A', '2,4%', 7]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>8,63%</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>8,23%</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>val</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>4,00</t>
-        </is>
-      </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>3,98</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>hist12</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr">
-        <is>
-          <t>{'b': 'IMA-B 5', 'l': ['2025-08', '2025-09', '2025-10', '2025-11', '2025-12', '2026-01', '2026-02', '2026-03', '2026-04', '2026-05', '2026-06', '2026-07', '2026-08'], 'f': [0.0, 1.64, 1.66, 3.1, 3.59, 5.89, 6.95, 6.67, 6.97, 7.26, 7.24, 8.41, 9.78], 'c': [0.0, 0.66, 1.69, 2.78, 3.76, 5.01, 6.29, 7.77, 9.19, 10.24, 10.48, 11.85, 13.28]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>histEnd</t>
-        </is>
-      </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>[12.94, 15.69, 'IMA-B 5']</t>
-        </is>
-      </c>
-      <c r="E214" t="inlineStr">
-        <is>
-          <t>[9.78, 13.28, 'IMA-B 5']</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr">
-        <is>
-          <t>comentario</t>
-        </is>
-      </c>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>['Em julho, os títulos de crédito indexados ao IPCA precificados pela ANBIMA apresentaram desempenho negativo, refletindo a elevação da curva real de juros ao longo do período. Embora os spreads de crédito tenham fechado cerca de 16 bps em relação ao mês anterior, o avanço da curva de juros reais prevaleceu sobre esse efeito.', 'No mercado primário, manteve-se o cenário de oferta restrita, com parcela relevante das emissões sendo absorvida pelos balanços dos bancos distribuidores. No secundário, houve retomada da demanda por papéis incentivados, inclusive nos vencimentos mais longos.', 'Do ponto de vista da gestão, mantivemos postura cautelosa, priorizando o encurtamento da duration da carteira como forma de mitigar volatilidade e reduzir a sensibilidade a movimentos adversos nos spreads.', 'O Infra Plus apresentou rentabilidade, isenta de imposto de renda, de &lt;b&gt;1,24%&lt;/b&gt; no mês, acumulando &lt;b&gt;7,80%&lt;/b&gt; no ano. Destacam-se as debêntures de RUMO e NTS, enquanto Alloha Fibra foi a maior detratora.']</t>
-        </is>
-      </c>
-      <c r="E215" t="inlineStr">
-        <is>
-          <t>['Em agosto, os títulos de crédito indexados ao IPCA precificados pela ANBIMA apresentaram desempenho positivo, refletindo principalmente o movimento de fechamento da curva real de juros observado ao longo do período. Embora os spreads de crédito tenham registrado abertura média de aproximadamente 5 bps em relação a julho, a redução das taxas reais ao longo da estrutura a termo mais do que compensou esse movimento. Como resultado, as taxas médias dos títulos incentivados precificados pela ANBIMA encerraram o mês com fechamento próximo de 16 bps, proporcionando valorização dos ativos no mercado secundário.', 'No mercado primário, manteve-se o cenário de oferta restrita de ativos, com parcela relevante das emissões sendo absorvida diretamente pelos balanços dos bancos distribuidores. Já no mercado secundário, observou-se um nível de liquidez inferior à média observada ao longo de 2025, contribuindo para um ambiente de maior equilíbrio entre oferta e demanda dos ativos negociados.', 'Sob a ótica da gestão, mantivemos uma postura cautelosa ao longo do período, priorizando o encurtamento da duration da carteira como forma de mitigar a volatilidade e reduzir a sensibilidade do portfólio a eventuais movimentos adversos nos spreads de crédito. Apesar da melhora observada no desempenho dos ativos incentivados no mês, seguimos avaliando que os níveis atuais de prêmio ainda oferecem pouca margem de segurança frente aos riscos inerentes à classe. Dessa forma, permanecemos atentos à evolução das condições de mercado e à dinâmica de precificação dos ativos, buscando identificar oportunidades mais atrativas para aumentar a exposição ao risco de crédito de forma gradual e criteriosa, quando a relação risco-retorno se mostrar mais favorável.', 'Nesse cenário, o Tivio Infra Plus apresentou rentabilidade, isenta de imposto de renda de 1,26% no mês, acumulando 5,98% no ano. Na atribuição de performance, pode-se destacar as debêntures de NTS e São Simão, enquanto as de Jalles Machado foram as maiores detratoras.']</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="E216" t="inlineStr">
-        <is>
-          <t>31/08/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>Julho de 2026</t>
-        </is>
-      </c>
-      <c r="E217" t="inlineStr">
-        <is>
-          <t>Agosto de 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>julho de 2026</t>
-        </is>
-      </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>agosto de 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>Julho 2026</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>Agosto 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>-jul26</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>-ago26</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>julho/2026</t>
-        </is>
-      </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>agosto/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>data</t>
-        </is>
-      </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>const A=6;const track</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>const A=7;const track</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>libs de exportação</t>
-        </is>
-      </c>
-      <c r="D223" t="inlineStr">
-        <is>
-          <t>CDN</t>
-        </is>
-      </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>4 referências → vendor/ local (CDN como reserva)</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>s1</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="D224" t="inlineStr">
-        <is>
-          <t>Julho 2026</t>
-        </is>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>Agosto 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>s2</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>Julho 2026</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>Agosto 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>s8</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>Julho 2026</t>
-        </is>
-      </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>Agosto 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>r1</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>Julho 2026</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>Agosto 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>e1</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>Julho 2026</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>Agosto 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>r1</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>Relatórios de Gestão · Crédito Privado</t>
-        </is>
-      </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>Gerador de Relatório de Gestão · Crédito Privado</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>r1</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>desc</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>Relatório completo de 4 páginas (A4) por fundo, Banks, Institucional, Institucional 15, Institucional 30 e Infra Plus: objetivo, rentabilidade, emissores, alocação e rating; histórico e comentário do gestor; mercado de crédito; e características + disclaimer. Exportação em JPG e PDF.</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório completo de 4 páginas (A4) por fundo, Banks, Institucional, Institucional 15, Institucional 30 e Infra Plus: objetivo, rentabilidade, emissores, alocação e rating; histórico e comentário do gestor; mercado de crédito; e características + disclaimer. Exportação em JPG e PDF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>r2</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>Relatório de Gestão · Incentivado CDI 30</t>
-        </is>
-      </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>Gerador de Relatório de Gestão · Incentivado CDI 30</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>r2</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>desc</t>
-        </is>
-      </c>
-      <c r="D232" t="inlineStr">
-        <is>
-          <t>Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
-        </is>
-      </c>
-      <c r="E232" t="inlineStr">
-        <is>
-          <t>Construtor interativo, folha a folha. Os relatórios prontos do mês estão no card acima. Relatório de gestão mensal do Tivio Institucional Inc CDI 30 FIF (debêntures incentivadas · CDI).</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
-      </c>
-      <c r="D233" t="inlineStr">
-        <is>
-          <t>cards de relatório</t>
-        </is>
-      </c>
-      <c r="E233" t="inlineStr">
-        <is>
-          <t>2 registrados para Agosto 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>data automática</t>
-        </is>
-      </c>
-      <c r="D234" t="inlineStr"/>
-      <c r="E234" t="inlineStr">
         <is>
           <t>DATA_BASE=2026-08-31</t>
         </is>
@@ -13443,7 +11472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -13480,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>832184</v>
+        <v>833662</v>
       </c>
     </row>
     <row r="3">
@@ -13495,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>47637</v>
+        <v>1923065</v>
       </c>
     </row>
     <row r="4">
@@ -13510,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>838500</v>
+        <v>839985</v>
       </c>
     </row>
     <row r="5">
@@ -13525,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>47824</v>
+        <v>1927590</v>
       </c>
     </row>
     <row r="6">
@@ -13540,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>842446</v>
+        <v>843920</v>
       </c>
     </row>
     <row r="7">
@@ -13555,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>47848</v>
+        <v>1946164</v>
       </c>
     </row>
     <row r="8">
@@ -13570,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>840983</v>
+        <v>842461</v>
       </c>
     </row>
     <row r="9">
@@ -13585,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>47696</v>
+        <v>1919224</v>
       </c>
     </row>
     <row r="10">
@@ -13600,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>791785</v>
+        <v>793274</v>
       </c>
     </row>
     <row r="11">
@@ -13615,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46722</v>
+        <v>1560554</v>
       </c>
     </row>
     <row r="12">
@@ -13630,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>823202</v>
+        <v>824673</v>
       </c>
     </row>
     <row r="13">
@@ -13645,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>47651</v>
+        <v>1897910</v>
       </c>
     </row>
     <row r="14">
@@ -13660,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>832443</v>
+        <v>833914</v>
       </c>
     </row>
     <row r="15">
@@ -13675,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>47697</v>
+        <v>1916306</v>
       </c>
     </row>
     <row r="16">
@@ -13690,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>625363</v>
+        <v>626351</v>
       </c>
     </row>
     <row r="17">
@@ -13705,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>43631</v>
+        <v>305920</v>
       </c>
     </row>
     <row r="18">
@@ -13720,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>624108</v>
+        <v>625115</v>
       </c>
     </row>
     <row r="19">
@@ -13735,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>43545</v>
+        <v>287034</v>
       </c>
     </row>
     <row r="20">
@@ -13750,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>625103</v>
+        <v>626121</v>
       </c>
     </row>
     <row r="21">
@@ -13765,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42429</v>
+        <v>283919</v>
       </c>
     </row>
     <row r="22">
@@ -13780,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>832111</v>
+        <v>833629</v>
       </c>
     </row>
     <row r="23">
@@ -13795,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>47118</v>
+        <v>1909635</v>
       </c>
     </row>
     <row r="24">
@@ -13810,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>797583</v>
+        <v>793857</v>
       </c>
     </row>
     <row r="25">
@@ -13825,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>46717</v>
+        <v>1560004</v>
       </c>
     </row>
     <row r="26">
@@ -13840,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>840434</v>
+        <v>835600</v>
       </c>
     </row>
     <row r="27">
@@ -13855,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>47685</v>
+        <v>1919014</v>
       </c>
     </row>
     <row r="28">
@@ -13870,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3218147</v>
+        <v>3239620</v>
       </c>
     </row>
     <row r="29">
@@ -13885,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060312</v>
+        <v>1060313</v>
       </c>
     </row>
     <row r="30">
@@ -13981,7 +12010,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>tivio-relatorio-gestao-credito-privado.html</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -13990,22 +12019,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>122525</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>66613</v>
+        <v>65870</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AutomaTivio: ALT Light no desenho do relatório publicado
- ALT Light: razão social "TIVIO ALT LIGHT XP PREV", paleta própria no
  treemap (treemap_cores), 15 setores em linhas compactas com valor em azul
  (setores_max_relatorio, estrategia_linha).
- Caixa "Rentabilidade CDI +": período sem número (fundo sem 12M) sai.
- Gráfico do Estruturado: grade até o degrau abaixo do valor final, com
  folga para a linha e a etiqueta; mês de início parcial sem rótulo e a
  linha nascendo em 0 (vale para ALT 180, 90 e Light, como os publicados).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>843920</v>
+        <v>843923</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1946164</v>
+        <v>1945550</v>
       </c>
     </row>
     <row r="8">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>626351</v>
+        <v>626383</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>305920</v>
+        <v>302078</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>625115</v>
+        <v>625093</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>287034</v>
+        <v>287505</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>626121</v>
+        <v>626284</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>283919</v>
+        <v>283711</v>
       </c>
     </row>
     <row r="22">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3239620</v>
+        <v>3239874</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060313</v>
+        <v>1060177</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: Mercado de Crédito preenche a folha, caixa do T na tela, logos do e-mail menores
- Mercado de Crédito: com poucos setores (tabela IPCA) o painel ocupa a
  altura livre até a nota e as linhas crescem; o total da tabela larga em
  corpo menor para os números não encostarem.
- Caixa do T: sai a regra antiga do relatorio_vertical.html que a deixava
  transparente na tela e na exportação PNG/JPG.
- E-mail: logos em 30 px (Crédito Privado) e 44 px (ALT).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>833662</v>
+        <v>833143</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1923065</v>
+        <v>1906738</v>
       </c>
     </row>
     <row r="4">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>839985</v>
+        <v>839467</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1927590</v>
+        <v>1911437</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>843923</v>
+        <v>843406</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1945550</v>
+        <v>1928988</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>842461</v>
+        <v>841944</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1919224</v>
+        <v>1903123</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>793274</v>
+        <v>812058</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1560554</v>
+        <v>1901979</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>824673</v>
+        <v>824156</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1897910</v>
+        <v>1881925</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>833914</v>
+        <v>833399</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1916306</v>
+        <v>1900669</v>
       </c>
     </row>
     <row r="16">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>833629</v>
+        <v>833112</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1909635</v>
+        <v>1893613</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>793857</v>
+        <v>812654</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1560004</v>
+        <v>1900777</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>835600</v>
+        <v>835083</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1919014</v>
+        <v>1903091</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3239874</v>
+        <v>3240157</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060177</v>
+        <v>1060460</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: histórico em ECharts com acumulado; comentário ajustado e centralizado; T na exportação; Central conectada
- Rentabilidade histórica em ECharts (svg) com a mesma especificação do SVG
  do servidor e o acumulado no fim de cada linha, nas duas verticais.
- Comentário do gestor: texto curto cresce até o teto e fica centralizado
  na caixa; texto longo diminui até caber.
- Mercado de Crédito: vidro em tons de azul.
- ALT: rótulo "Taxa global".
- Caixa do T: chanfro feito com borda (o html2canvas ignorava clip-path) e
  folha com canto reto — a ponta não sai mais cortada no PNG/JPG/PDF baixado.
- Central: botão de volta no e-mail Nordea e saida/AAAA-MM/index.html como
  porta de entrada.
- Saída de agosto regenerada com os comentários de agosto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11472,7 +11472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>833143</v>
+        <v>837374</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1906738</v>
+        <v>1954048</v>
       </c>
     </row>
     <row r="4">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>839467</v>
+        <v>844142</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1911437</v>
+        <v>1967345</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>843406</v>
+        <v>848407</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1928988</v>
+        <v>1982981</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>841944</v>
+        <v>844766</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1903123</v>
+        <v>1962152</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>812058</v>
+        <v>815775</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1901979</v>
+        <v>1947337</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>824156</v>
+        <v>826969</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1881925</v>
+        <v>1928179</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>833399</v>
+        <v>836891</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1900669</v>
+        <v>1954540</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>626383</v>
+        <v>624863</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>302078</v>
+        <v>300733</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>625093</v>
+        <v>623155</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>287505</v>
+        <v>286918</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>626284</v>
+        <v>624241</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>283711</v>
+        <v>276744</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>833112</v>
+        <v>835949</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1893613</v>
+        <v>1951625</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>812654</v>
+        <v>815817</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1900777</v>
+        <v>1948754</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>835083</v>
+        <v>838848</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1903091</v>
+        <v>1954799</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3240157</v>
+        <v>3254516</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1060460</v>
+        <v>1063789</v>
       </c>
     </row>
     <row r="30">
@@ -11959,7 +11959,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>50202</v>
+        <v>50469</v>
       </c>
     </row>
     <row r="33">
@@ -12020,6 +12020,21 @@
       </c>
       <c r="C36" t="n">
         <v>65870</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>index.html</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>390</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AutomaTivio: caixa do T quadrada (sem chanfro), 124x124 visíveis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>837374</v>
+        <v>837258</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1954048</v>
+        <v>1956523</v>
       </c>
     </row>
     <row r="4">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>844142</v>
+        <v>844020</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1967345</v>
+        <v>1964748</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>848407</v>
+        <v>848284</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1982981</v>
+        <v>1981590</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>844766</v>
+        <v>844652</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1962152</v>
+        <v>1956912</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>815775</v>
+        <v>815660</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1947337</v>
+        <v>1943110</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>826969</v>
+        <v>826844</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1928179</v>
+        <v>1932741</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>836891</v>
+        <v>836775</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1954540</v>
+        <v>1951967</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>624863</v>
+        <v>624735</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>300733</v>
+        <v>296512</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>623155</v>
+        <v>623070</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>286918</v>
+        <v>290770</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>624241</v>
+        <v>624141</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>276744</v>
+        <v>282399</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>835949</v>
+        <v>835834</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1951625</v>
+        <v>1953536</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>815817</v>
+        <v>815847</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1948754</v>
+        <v>1948140</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>838848</v>
+        <v>838865</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1954799</v>
+        <v>1955192</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3254516</v>
+        <v>3254251</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1063789</v>
+        <v>1063524</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: página 1 conforme o tamanho das listas; tabela de spreads com respiro; razão social do Banks
- Banks: razão social "TIVIO BANKS RENDA FIXA CRÉDITO PRIVADO FIF – RL".
- Página 1 do high grade: emissores, rating e setores ocupam a folha até o
  rodapé; lista curta espaça as linhas (com teto) e engrossa a barra.
- Mercado de Crédito: colunas redistribuídas (%, Variação e Duration com
  folga), célula centrada na vertical, total em 17 px; linha mínima de 32 px
  para a tabela de 23 setores caber no painel sem espremer o fim.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -4750,7 +4750,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2 registrados para Agosto 2026</t>
+          <t>1 registrados para Agosto 2026</t>
         </is>
       </c>
     </row>
@@ -4788,12 +4788,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -4822,34 +4822,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>infraplus</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus</t>
+          <t>Tivio Banks</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>carteira</t>
+          <t>números no comentário</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>linhas sem data na Base Carteira — a alocação exibida pode ser de outro mês; conferir a coluna Data da planilha</t>
+          <t>o texto cita 10,54% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>banks</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tivio ALT 180</t>
+          <t>Tivio Banks</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4866,66 +4866,594 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>alt90</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tivio ALT 90</t>
+          <t>Tivio Institucional</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>comentário</t>
+          <t>números no comentário</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+          <t>o texto cita 10,44%, 95% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>institucional</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Top Gestor Ações Long Only</t>
+          <t>Tivio Institucional</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>% do benchmark (mes)</t>
+          <t>comentário</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>370% fora da faixa 0–300% — conferir unidade ou sinal do benchmark</t>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>inst15</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tivio Institucional 15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>o texto cita 10,73% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>inst15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tivio Institucional 15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>inst30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tivio Institucional 30</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>o texto cita 10,65% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>inst30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tivio Institucional 30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>infraplus</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>carteira</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>linhas sem data na Base Carteira — a alocação exibida pode ser de outro mês; conferir a coluna Data da planilha</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>infraplus</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>o texto cita 7,05% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>infraplus</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>bvp</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tivio BVP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>o texto cita 10,55% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>bvp</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tivio BVP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>rfcp</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tivio RF CP</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>o texto cita 93% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>rfcp</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tivio RF CP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>alt180</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>o texto cita 26,79%, 34,87% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>alt180</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>alt90</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>o texto cita 19,70% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>alt90</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>altlight</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>o texto cita 19,70% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>altlight</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>topgestorlongonly</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Top Gestor Ações Long Only</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>% do benchmark (mes)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>370% fora da faixa 0–300% — conferir unidade ou sinal do benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>infrapluscdi</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>o texto cita 8,64%, 82% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>infrapluscdi</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>esplanada</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Tivio Esplanada</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>carteira</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>linhas sem data na Base Carteira — a alocação exibida pode ser de outro mês; conferir a coluna Data da planilha</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>o texto cita 7,17% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>esplanada</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>números no comentário</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>o texto cita 10,03% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>comentário</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
         </is>
       </c>
     </row>
@@ -4940,7 +5468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -4974,12 +5502,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>altlight</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tivio ALT Light</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4996,12 +5524,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5018,12 +5546,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5040,56 +5568,56 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>BV Top Gestor Macro</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>sem cotas na dados_mensais</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>topgestorlongonly</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BV Top Gestor Macro</t>
+          <t>Top Gestor Ações Long Only</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>comentário do gestor</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não preenchido no arquivo de comentários</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top Gestor Ações Long Only</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5106,12 +5634,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5128,12 +5656,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>prevlowvol</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Prev Low Vol Itaú</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5150,42 +5678,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>atuarial</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio Atuarial</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
-        <is>
-          <t>não preenchido no arquivo de comentários</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>atuarial</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Tivio Atuarial</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>rentabilidade</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
         <is>
           <t>sem cotas na dados_mensais</t>
         </is>
@@ -11266,7 +11772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11362,100 +11868,49 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>relatorio/bvp</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é agosto</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>relatorio/atuarial</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>atuarial</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>relatório não gerado: sem dados nesta edição</t>
+          <t>sem dados — rentabilidade e PL mantidos</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>relatorio/credito_privado</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>bvp</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
-        <is>
-          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>tivio-email-fundos-credito.html</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>alt180</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é agosto</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>tivio-post-investment-solutions.html</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>topgestormacro</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -11472,7 +11927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -11500,7 +11955,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tivio Banks - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>Tivio Institucional 30 - Relatório de Gestão - Agosto 2026.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -11509,531 +11964,156 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>837258</v>
+        <v>840762</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tivio Banks - Relatório de Gestão - Agosto 2026.pptx</t>
+          <t>Tivio Esplanada - Relatório de Gestão - Agosto 2026.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1956523</v>
+        <v>814983</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tivio Institucional - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>Relatório de Gestão - Crédito Privado - Agosto 2026.html</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>844020</v>
+        <v>719736</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tivio Institucional - Relatório de Gestão - Agosto 2026.pptx</t>
+          <t>tivio-construtor-one-pager.html</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1964748</v>
+        <v>88026</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15 - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>tivio-email-fundos-credito.html</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>848284</v>
+        <v>176798</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15 - Relatório de Gestão - Agosto 2026.pptx</t>
+          <t>tivio-email-nordea-studio.html</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1981590</v>
+        <v>50469</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>tivio-post-credito-estruturado.html</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>844652</v>
+        <v>114702</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Agosto 2026.pptx</t>
+          <t>tivio-post-credito-privado.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1956912</v>
+        <v>127504</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>tivio-post-investment-solutions.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>815660</v>
+        <v>105529</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tivio Infra Plus - Relatório de Gestão - Agosto 2026.pptx</t>
+          <t>tivio-central.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>pptx</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1943110</v>
+        <v>65182</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tivio BVP - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>html</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>826844</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Tivio BVP - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>1932741</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Tivio RF CP - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>836775</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Tivio RF CP - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1951967</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180 - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>624735</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180 - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>296512</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90 - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>623070</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90 - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>290770</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>624141</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>282399</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>835834</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>1953536</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>815847</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>1948140</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev - Relatório de Gestão - Agosto 2026.pdf</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>pdf</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>838865</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev - Relatório de Gestão - Agosto 2026.pptx</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>pptx</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1955192</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Relatório de Gestão - Crédito Privado - Agosto 2026.html</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>3254251</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Relatório de Gestão - Crédito Estruturado - Agosto 2026.html</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>1063524</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>tivio-construtor-one-pager.html</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>88026</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>tivio-email-fundos-credito.html</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>176798</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>tivio-email-nordea-studio.html</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>50469</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>tivio-post-credito-estruturado.html</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>114702</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>tivio-post-credito-privado.html</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>127504</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>tivio-post-investment-solutions.html</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>105529</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>tivio-central.html</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>65870</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>index.html</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
         <v>390</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: "Data base:" sob a tabela de rentabilidade em todos os fundos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -4750,7 +4750,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>1 registrados para Agosto 2026</t>
+          <t>2 registrados para Agosto 2026</t>
         </is>
       </c>
     </row>
@@ -4788,12 +4788,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -4822,34 +4822,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>infraplus</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tivio Banks</t>
+          <t>Tivio Infra Plus</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>números no comentário</t>
+          <t>carteira</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>o texto cita 10,54% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+          <t>linhas sem data na Base Carteira — a alocação exibida pode ser de outro mês; conferir a coluna Data da planilha</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>banks</t>
+          <t>alt180</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tivio Banks</t>
+          <t>Tivio ALT 180</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4866,594 +4866,66 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>alt90</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tivio Institucional</t>
+          <t>Tivio ALT 90</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>números no comentário</t>
+          <t>comentário</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>o texto cita 10,44%, 95% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
+          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>institucional</t>
+          <t>topgestorlongonly</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tivio Institucional</t>
+          <t>Top Gestor Ações Long Only</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>comentário</t>
+          <t>% do benchmark (mes)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
+          <t>370% fora da faixa 0–300% — conferir unidade ou sinal do benchmark</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>inst15</t>
+          <t>esplanada</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tivio Institucional 15</t>
+          <t>Tivio Esplanada</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>números no comentário</t>
+          <t>carteira</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>o texto cita 10,73% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>inst15</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Tivio Institucional 15</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Tivio Institucional 30</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>o texto cita 10,65% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>inst30</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Tivio Institucional 30</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>carteira</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
           <t>linhas sem data na Base Carteira — a alocação exibida pode ser de outro mês; conferir a coluna Data da planilha</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>o texto cita 7,05% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>infraplus</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>bvp</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Tivio BVP</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>o texto cita 10,55% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>bvp</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Tivio BVP</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>rfcp</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Tivio RF CP</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>o texto cita 93% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>rfcp</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Tivio RF CP</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>alt180</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>o texto cita 26,79%, 34,87% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>alt180</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Tivio ALT 180</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>alt90</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>o texto cita 19,70% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>alt90</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Tivio ALT 90</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>altlight</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>o texto cita 19,70% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>altlight</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Tivio ALT Light</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>topgestorlongonly</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Top Gestor Ações Long Only</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>% do benchmark (mes)</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>370% fora da faixa 0–300% — conferir unidade ou sinal do benchmark</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>infrapluscdi</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>o texto cita 8,64%, 82% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>infrapluscdi</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Tivio Infra Plus CDI</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>esplanada</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>carteira</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>linhas sem data na Base Carteira — a alocação exibida pode ser de outro mês; conferir a coluna Data da planilha</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>esplanada</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>o texto cita 7,17% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>esplanada</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Tivio Esplanada</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>legacy</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>números no comentário</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>o texto cita 10,03% — nenhum bate com um valor calculado deste fundo nesta edição. Conferir se o texto é do mês certo (o sistema não altera o texto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>legacy</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Tivio Legacy Prev</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>comentário</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>o texto se refere a "setembro" como o mês corrente — a data base é agosto/2026. Conferir se o comentário é o desta edição.</t>
         </is>
       </c>
     </row>
@@ -5468,7 +4940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -5502,12 +4974,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>topgestor</t>
+          <t>altlight</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BV Top Gestor Crédito Privado</t>
+          <t>Tivio ALT Light</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5524,12 +4996,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>topgestorhy</t>
+          <t>topgestor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tivio Top Gestor HY</t>
+          <t>BV Top Gestor Crédito Privado</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5546,12 +5018,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>topgestorativo</t>
+          <t>topgestorhy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BV Top Gestor RF Ativo</t>
+          <t>Tivio Top Gestor HY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5568,56 +5040,56 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>topgestorativo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BV Top Gestor Macro</t>
+          <t>BV Top Gestor RF Ativo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>rentabilidade</t>
+          <t>comentário do gestor</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>sem cotas na dados_mensais</t>
+          <t>não preenchido no arquivo de comentários</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>topgestorlongonly</t>
+          <t>topgestormacro</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Top Gestor Ações Long Only</t>
+          <t>BV Top Gestor Macro</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>comentário do gestor</t>
+          <t>rentabilidade</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>não preenchido no arquivo de comentários</t>
+          <t>sem cotas na dados_mensais</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>topmanagerglobal</t>
+          <t>topgestorlongonly</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tivio Top Manager Global</t>
+          <t>Top Gestor Ações Long Only</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5634,12 +5106,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ativorf</t>
+          <t>topmanagerglobal</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tivio RF Ativo Longo Prazo</t>
+          <t>Tivio Top Manager Global</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5656,12 +5128,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>prevlowvol</t>
+          <t>ativorf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tivio Prev Low Vol Itaú</t>
+          <t>Tivio RF Ativo Longo Prazo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5678,20 +5150,42 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>prevlowvol</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tivio Prev Low Vol Itaú</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>comentário do gestor</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>não preenchido no arquivo de comentários</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>atuarial</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Tivio Atuarial</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>rentabilidade</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>sem cotas na dados_mensais</t>
         </is>
@@ -11772,7 +11266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11868,49 +11362,100 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>relatorio/bvp</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>alt180</t>
+          <t>bvp</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>o texto se refere a "julho" como o mês corrente — a data base é agosto</t>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>relatorio/atuarial</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>topgestormacro</t>
+          <t>atuarial</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>sem dados — rentabilidade e PL mantidos</t>
+          <t>relatório não gerado: sem dados nesta edição</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>relatorio/credito_privado</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>bvp</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>logo não encontrado em assets/logos (procurei "tivio_bvp")</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tivio-email-fundos-credito.html</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>alt180</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>o texto se refere a "julho" como o mês corrente — a data base é agosto</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>topgestormacro</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>sem dados — rentabilidade e PL mantidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>tivio-central.html</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>card "Gerador de Relatório de Gestão · Incentivado CDI 30" removido: aponta para "Tivio Incentivado CDI 30 - Relatório de Gestão Mensal.html", que não existe nesta edição</t>
         </is>
@@ -11927,7 +11472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -11955,7 +11500,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tivio Institucional 30 - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>Tivio Banks - Relatório de Gestão - Agosto 2026.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -11964,156 +11509,531 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>840762</v>
+        <v>837689</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tivio Esplanada - Relatório de Gestão - Agosto 2026.pdf</t>
+          <t>Tivio Banks - Relatório de Gestão - Agosto 2026.pptx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>814983</v>
+        <v>1962279</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Relatório de Gestão - Crédito Privado - Agosto 2026.html</t>
+          <t>Tivio Institucional - Relatório de Gestão - Agosto 2026.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>719736</v>
+        <v>844461</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tivio-construtor-one-pager.html</t>
+          <t>Tivio Institucional - Relatório de Gestão - Agosto 2026.pptx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>88026</v>
+        <v>1969668</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tivio-email-fundos-credito.html</t>
+          <t>Tivio Institucional 15 - Relatório de Gestão - Agosto 2026.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>176798</v>
+        <v>848724</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tivio-email-nordea-studio.html</t>
+          <t>Tivio Institucional 15 - Relatório de Gestão - Agosto 2026.pptx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50469</v>
+        <v>1987504</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tivio-post-credito-estruturado.html</t>
+          <t>Tivio Institucional 30 - Relatório de Gestão - Agosto 2026.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>114702</v>
+        <v>845108</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tivio-post-credito-privado.html</t>
+          <t>Tivio Institucional 30 - Relatório de Gestão - Agosto 2026.pptx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>127504</v>
+        <v>1963344</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tivio-post-investment-solutions.html</t>
+          <t>Tivio Infra Plus - Relatório de Gestão - Agosto 2026.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>105529</v>
+        <v>816001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tivio-central.html</t>
+          <t>Tivio Infra Plus - Relatório de Gestão - Agosto 2026.pptx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>html</t>
+          <t>pptx</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>65182</v>
+        <v>1947425</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Tivio BVP - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>827327</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tivio BVP - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1942080</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tivio RF CP - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>837221</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tivio RF CP - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1959817</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>624550</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tivio ALT 180 - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>296383</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90 - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>622922</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tivio ALT 90 - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>290733</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>624149</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tivio ALT Light - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>282447</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>836306</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tivio Infra Plus CDI - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1959835</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>816045</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tivio Esplanada - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1952312</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev - Relatório de Gestão - Agosto 2026.pdf</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>839195</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tivio Legacy Prev - Relatório de Gestão - Agosto 2026.pptx</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pptx</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1962176</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão - Crédito Privado - Agosto 2026.html</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3256183</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Relatório de Gestão - Crédito Estruturado - Agosto 2026.html</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1064610</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tivio-construtor-one-pager.html</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>88026</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tivio-email-fundos-credito.html</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>176798</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tivio-email-nordea-studio.html</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>50469</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>tivio-post-credito-estruturado.html</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>114702</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tivio-post-credito-privado.html</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>127504</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>tivio-post-investment-solutions.html</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>105529</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>tivio-central.html</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>65870</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>html</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C37" t="n">
         <v>390</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: razão social e CNPJ dos fundos de Crédito Privado
- configs/fundos.yml: razao_social de Institucional, Institucional 15,
  Infra Plus, Infra Plus CDI, Esplanada, Legacy e RF CP.
- Legacy: cnpj_exibido 09.166.056/0001-95 no cabeçalho (a DePara tem
  09.083.848/0001-04, que segue sendo usado para buscar as taxas).
- Cabeçalho: a linha da razão social diminui o corpo conforme o tamanho,
  para caber numa linha até o fim do traço.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>837689</v>
+        <v>837819</v>
       </c>
     </row>
     <row r="3">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>844461</v>
+        <v>844468</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1969668</v>
+        <v>1969672</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>848724</v>
+        <v>848655</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1987504</v>
+        <v>1987498</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>845108</v>
+        <v>845128</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1963344</v>
+        <v>1963705</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>816001</v>
+        <v>816180</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1947425</v>
+        <v>1947270</v>
       </c>
     </row>
     <row r="12">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>837221</v>
+        <v>837261</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1959817</v>
+        <v>1959832</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>624550</v>
+        <v>624721</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296383</v>
+        <v>296512</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>622922</v>
+        <v>623060</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290733</v>
+        <v>290770</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>624149</v>
+        <v>624139</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>282447</v>
+        <v>282399</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>836306</v>
+        <v>836366</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1959835</v>
+        <v>1959857</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>816045</v>
+        <v>816368</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1952312</v>
+        <v>1952568</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>839195</v>
+        <v>839489</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1962176</v>
+        <v>1960320</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3256183</v>
+        <v>3256574</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1064610</v>
+        <v>1064688</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: setores com poucas linhas (Banks) ocupam a coluna, como no publicado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>837819</v>
+        <v>837841</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1962279</v>
+        <v>1962211</v>
       </c>
     </row>
     <row r="4">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296512</v>
+        <v>296383</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>623060</v>
+        <v>622912</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290770</v>
+        <v>290733</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>624139</v>
+        <v>624147</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>282399</v>
+        <v>282447</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>836366</v>
+        <v>836369</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1959857</v>
+        <v>1959851</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>816368</v>
+        <v>816222</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1952568</v>
+        <v>1952396</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>839489</v>
+        <v>839350</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1960320</v>
+        <v>1960537</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3256574</v>
+        <v>3256752</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1064688</v>
+        <v>1064858</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: Esplanada com a 3a linha Bench Tributado (IMA-B 5 x 0,85) no histórico
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296383</v>
+        <v>296512</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>622912</v>
+        <v>623060</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290733</v>
+        <v>290770</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>624147</v>
+        <v>624139</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>282447</v>
+        <v>282399</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>836369</v>
+        <v>836366</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1959851</v>
+        <v>1959857</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>816222</v>
+        <v>838809</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1952396</v>
+        <v>1968601</v>
       </c>
     </row>
     <row r="26">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3256752</v>
+        <v>3258241</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1064858</v>
+        <v>1065251</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: Destaques e e-mails exportados pelo Python; guia de processos
- exporters/destaques.py: JPG 2160x2880 de cada página dos três carrosséis
  e um pacote PDF por carrossel (1080x1440 pt, 4x), em
  saida/AAAA-MM/destaques/<vertical>/, numerados na ordem do carrossel.
- exporters/emails.py: as quatro versões do e-mail (Ágora, BTG, XP,
  Quadrado) com PNG de cada card, PNG do e-mail completo e o HTML de
  disparo, em saida/AAAA-MM/emails/<versao>/.
- As duas exportações chamam as mesmas funções dos botões das páginas.
- configs/edicao.yml: saidas.destaques e saidas.emails.
- Documentacao_AutomaTivio/COMO_FUNCIONA.md: o que cada processo faz,
  entradas, saídas, onde mexer e checklist.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11472,7 +11472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1969672</v>
+        <v>1969569</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>848655</v>
+        <v>848514</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1987498</v>
+        <v>1987494</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>845128</v>
+        <v>844982</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1963705</v>
+        <v>1963839</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>816180</v>
+        <v>816073</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1947270</v>
+        <v>1947306</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>827327</v>
+        <v>827186</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1942080</v>
+        <v>1942156</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>837261</v>
+        <v>837128</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1959832</v>
+        <v>1959089</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>624721</v>
+        <v>624536</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296512</v>
+        <v>296383</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>623060</v>
+        <v>622912</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290770</v>
+        <v>290733</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>624139</v>
+        <v>624147</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>282399</v>
+        <v>282447</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>836366</v>
+        <v>836369</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1959857</v>
+        <v>1959851</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>838809</v>
+        <v>838521</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968601</v>
+        <v>1968814</v>
       </c>
     </row>
     <row r="26">
@@ -12025,15 +12025,45 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>destaques</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>jpg</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>emails</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>html</t>
         </is>
       </c>
-      <c r="C37" t="n">
+      <c r="C39" t="n">
         <v>390</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AutomaTivio: taxas juntas à esquerda e patrimônios juntos à direita nas Características gerais
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>837841</v>
+        <v>837852</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1962211</v>
+        <v>1962146</v>
       </c>
     </row>
     <row r="4">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>844468</v>
+        <v>844475</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1969569</v>
+        <v>1969655</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>848514</v>
+        <v>848666</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1987494</v>
+        <v>1987683</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>844982</v>
+        <v>845139</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1963839</v>
+        <v>1963695</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>816073</v>
+        <v>816194</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1947306</v>
+        <v>1947219</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>827186</v>
+        <v>827340</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1942156</v>
+        <v>1942019</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>837128</v>
+        <v>837278</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1959089</v>
+        <v>1959870</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>624536</v>
+        <v>624730</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296383</v>
+        <v>296504</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>622912</v>
+        <v>623076</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290733</v>
+        <v>290714</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>624147</v>
+        <v>624156</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>282447</v>
+        <v>282324</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>836369</v>
+        <v>836377</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1959851</v>
+        <v>1959922</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>838521</v>
+        <v>838819</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968814</v>
+        <v>1968614</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>839350</v>
+        <v>839500</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1960537</v>
+        <v>1960279</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3258241</v>
+        <v>3258333</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1065251</v>
+        <v>1065343</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: selo "Rating S&P / brAMP1" nos relatórios e no one-pager, como nos posts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>837852</v>
+        <v>837832</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1962146</v>
+        <v>1962136</v>
       </c>
     </row>
     <row r="4">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>844475</v>
+        <v>844455</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1969655</v>
+        <v>1969646</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>848666</v>
+        <v>848644</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1987683</v>
+        <v>1987673</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>845139</v>
+        <v>845141</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1963695</v>
+        <v>1963689</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>816194</v>
+        <v>816089</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1947219</v>
+        <v>1947249</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>827340</v>
+        <v>827201</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1942019</v>
+        <v>1942090</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>837278</v>
+        <v>837147</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1959870</v>
+        <v>1959121</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>624730</v>
+        <v>624532</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296504</v>
+        <v>296368</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>623076</v>
+        <v>622912</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290714</v>
+        <v>290671</v>
       </c>
     </row>
     <row r="20">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>282324</v>
+        <v>282366</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>836377</v>
+        <v>836383</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1959922</v>
+        <v>1959909</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>838819</v>
+        <v>838535</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968614</v>
+        <v>1968819</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>839500</v>
+        <v>839366</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1960279</v>
+        <v>1960489</v>
       </c>
     </row>
     <row r="28">
@@ -11929,7 +11929,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>88026</v>
+        <v>88025</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
AutomaTivio: disclaimer dos relatórios vira "MATERIAL TÉCNICO" com o texto novo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>837832</v>
+        <v>832380</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1962136</v>
+        <v>1961068</v>
       </c>
     </row>
     <row r="4">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>844455</v>
+        <v>839113</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1969646</v>
+        <v>1968576</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>848644</v>
+        <v>843397</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1987673</v>
+        <v>1986603</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>845141</v>
+        <v>839298</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1963689</v>
+        <v>1962582</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>816089</v>
+        <v>810307</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1947249</v>
+        <v>1946106</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>827201</v>
+        <v>821525</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1942090</v>
+        <v>1940905</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>837147</v>
+        <v>831499</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1959121</v>
+        <v>1958756</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>624532</v>
+        <v>618635</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>296368</v>
+        <v>295387</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>622912</v>
+        <v>616882</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>290671</v>
+        <v>289597</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>624156</v>
+        <v>617948</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>282366</v>
+        <v>281206</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>836383</v>
+        <v>830443</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1959909</v>
+        <v>1958809</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>838535</v>
+        <v>832990</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1968819</v>
+        <v>1967496</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>839366</v>
+        <v>833734</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1960489</v>
+        <v>1959166</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3258333</v>
+        <v>3231313</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1065343</v>
+        <v>1057237</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: taxa do Legacy pelo CNPJ publicado; SAC e Ouvidoria no corpo do disclaimer
- Taxa e performance são buscadas pelo cnpj_exibido quando ele existe: no
  Legacy o CNPJ da DePara é outra classe, com taxa 0%; o publicado tem 0,50%.
- SAC e Ouvidoria acompanham o corpo do texto do disclaimer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11241,7 +11241,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,00% a.a.</t>
+          <t>0,50% a.a.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>832380</v>
+        <v>832189</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1961068</v>
+        <v>1961063</v>
       </c>
     </row>
     <row r="4">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>839113</v>
+        <v>838925</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1968576</v>
+        <v>1968568</v>
       </c>
     </row>
     <row r="6">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>843397</v>
+        <v>843208</v>
       </c>
     </row>
     <row r="7">
@@ -11584,7 +11584,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1986603</v>
+        <v>1986595</v>
       </c>
     </row>
     <row r="8">
@@ -11599,7 +11599,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>839298</v>
+        <v>839119</v>
       </c>
     </row>
     <row r="9">
@@ -11614,7 +11614,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1962582</v>
+        <v>1962573</v>
       </c>
     </row>
     <row r="10">
@@ -11629,7 +11629,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>810307</v>
+        <v>810134</v>
       </c>
     </row>
     <row r="11">
@@ -11644,7 +11644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1946106</v>
+        <v>1946096</v>
       </c>
     </row>
     <row r="12">
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>821525</v>
+        <v>821345</v>
       </c>
     </row>
     <row r="13">
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1940905</v>
+        <v>1940895</v>
       </c>
     </row>
     <row r="14">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>831499</v>
+        <v>831185</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1958756</v>
+        <v>1958003</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618635</v>
+        <v>618261</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>295387</v>
+        <v>295251</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>616882</v>
+        <v>616542</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>289597</v>
+        <v>289552</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>617948</v>
+        <v>617774</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>281206</v>
+        <v>281246</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830443</v>
+        <v>830272</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1958809</v>
+        <v>1958793</v>
       </c>
     </row>
     <row r="24">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832990</v>
+        <v>832511</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1967496</v>
+        <v>1967697</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>833734</v>
+        <v>833420</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959166</v>
+        <v>1959374</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3231313</v>
+        <v>3231558</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1057237</v>
+        <v>1057482</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
AutomaTivio: alocação real dos ALT pelo Book Maravi com de-para (visão da gestão)
- configs/fundos.yml: tabelas book_depara `alt` (ALT 90, ALT 180, HYD60) e
  `alt_light`; os percentuais dos books de mesmo rótulo são somados.
- ContextoFundo.alocacao_real: um corte só, usado pelo treemap do
  relatório e pelo post de Crédito Estruturado. Fundo sem book_depara segue
  no corte antigo (Tipo aj. + tipo_label).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 46.9}, {'n': 'FIDCs Cotas Mezanino', 'p': 27.0}, {'n': 'Bancário', 'p': 6.1}, {'n': 'Fiagro', 'p': 5.5}, {'n': 'Liquidez', 'p': 5.3}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Precatório', 'p': 2.7}, {'n': 'Crédito Estruturado', 'p': 2.6}]</t>
+          <t>[{'n': 'FIDC Sênior', 'p': 46.3}, {'n': 'FIDC Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 11.4}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatórios', 'p': 2.7}]</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDCs Cotas Sênior', 'p': 82.9}, {'n': 'Bancário', 'p': 8.3}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Fiagro', 'p': 2.9}, {'n': 'Liquidez', 'p': 1.9}, {'n': 'FIDCs Cotas Mezanino', 'p': 0.6}]</t>
+          <t>[{'n': 'FIDC Sênior', 'p': 81.4}, {'n': 'Liquidez', 'p': 10.2}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Crédito Estruturado', 'p': 2.9}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDC Mezanino', 'p': 0.6}]</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 40.7}, {'n': 'Crédito Privado', 'p': 25.8}, {'n': 'FIDCs Cotas Sênior', 'p': 23.5}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'Ações', 'p': 1.9}]</t>
+          <t>[{'n': 'Bancário', 'p': 40.7}, {'n': 'Crédito Privado', 'p': 25.8}, {'n': 'FIDC Sênior', 'p': 23.6}, {'n': 'Liquidez', 'p': 7.7}, {'n': 'Padrão', 'p': 2.0}]</t>
         </is>
       </c>
     </row>
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1968568</v>
+        <v>1968465</v>
       </c>
     </row>
     <row r="6">
@@ -11689,7 +11689,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>831185</v>
+        <v>831318</v>
       </c>
     </row>
     <row r="15">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1958003</v>
+        <v>1958746</v>
       </c>
     </row>
     <row r="16">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618261</v>
+        <v>618455</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>295251</v>
+        <v>295342</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>616542</v>
+        <v>616972</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>289552</v>
+        <v>289721</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>617774</v>
+        <v>617607</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>281246</v>
+        <v>281173</v>
       </c>
     </row>
     <row r="22">
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>830272</v>
+        <v>830269</v>
       </c>
     </row>
     <row r="23">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1958793</v>
+        <v>1958799</v>
       </c>
     </row>
     <row r="24">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1057482</v>
+        <v>1057406</v>
       </c>
     </row>
     <row r="30">
@@ -11974,7 +11974,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>114702</v>
+        <v>114655</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
AutomaTivio: alocação real com os nomes da gestão; book "Padrão" resolvido pelo tipo do ativo
- Rótulos: FIDCs Cota Sênior, FIDCs Cota Mezanino, Liquidez, Crédito
  Estruturado, Precatório, Fiagro.
- "Padrão" é posição sem book na planilha e nunca aparece: o tipo do ativo
  (Tipo aj.) decide o book (book_sem_book em fundos.yml) — ação ordinária
  vira FIP, LFT/Caixa vira Liquidez, FIDC Sr vira FIDCs Cota Sênior. ALT
  Light passa a fechar com o publicado: Liquidez 7,8% e FIP 1,9%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDC Sênior', 'p': 46.3}, {'n': 'FIDC Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 11.4}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatórios', 'p': 2.7}]</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 46.3}, {'n': 'FIDCs Cota Mezanino', 'p': 27.0}, {'n': 'Liquidez', 'p': 11.4}, {'n': 'Crédito Estruturado', 'p': 5.5}, {'n': 'Crédito Privado', 'p': 3.4}, {'n': 'Fiagro', 'p': 3.2}, {'n': 'Precatório', 'p': 2.7}]</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>[{'n': 'FIDC Sênior', 'p': 81.4}, {'n': 'Liquidez', 'p': 10.2}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Crédito Estruturado', 'p': 2.9}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDC Mezanino', 'p': 0.6}]</t>
+          <t>[{'n': 'FIDCs Cota Sênior', 'p': 81.4}, {'n': 'Liquidez', 'p': 10.2}, {'n': 'Crédito Privado', 'p': 3.6}, {'n': 'Crédito Estruturado', 'p': 2.9}, {'n': 'Fiagro', 'p': 1.5}, {'n': 'FIDCs Cota Mezanino', 'p': 0.6}]</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 40.7}, {'n': 'Crédito Privado', 'p': 25.8}, {'n': 'FIDC Sênior', 'p': 23.6}, {'n': 'Liquidez', 'p': 7.7}, {'n': 'Padrão', 'p': 2.0}]</t>
+          <t>[{'n': 'Bancário', 'p': 40.7}, {'n': 'Crédito Privado', 'p': 25.8}, {'n': 'FIDCs Cota Sênior', 'p': 23.5}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
         </is>
       </c>
     </row>
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>832189</v>
+        <v>832315</v>
       </c>
     </row>
     <row r="3">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>838925</v>
+        <v>838802</v>
       </c>
     </row>
     <row r="5">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1968465</v>
+        <v>1968568</v>
       </c>
     </row>
     <row r="6">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618455</v>
+        <v>618536</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>295342</v>
+        <v>295318</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>616972</v>
+        <v>616870</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>289721</v>
+        <v>289653</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>617607</v>
+        <v>617753</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>281173</v>
+        <v>281200</v>
       </c>
     </row>
     <row r="22">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>832511</v>
+        <v>832799</v>
       </c>
     </row>
     <row r="25">
@@ -11854,7 +11854,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1967697</v>
+        <v>1967484</v>
       </c>
     </row>
     <row r="26">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>833420</v>
+        <v>833559</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959374</v>
+        <v>1959157</v>
       </c>
     </row>
     <row r="28">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1057406</v>
+        <v>1057479</v>
       </c>
     </row>
     <row r="30">
@@ -11974,7 +11974,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>114655</v>
+        <v>114680</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
AutomaTivio: book Deb sai como Debêntures na alocação real dos ALT
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>[{'n': 'Bancário', 'p': 40.7}, {'n': 'Crédito Privado', 'p': 25.8}, {'n': 'FIDCs Cota Sênior', 'p': 23.5}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
+          <t>[{'n': 'Bancário', 'p': 40.7}, {'n': 'Debêntures', 'p': 25.8}, {'n': 'FIDCs Cota Sênior', 'p': 23.5}, {'n': 'Liquidez', 'p': 7.8}, {'n': 'FIP', 'p': 1.9}]</t>
         </is>
       </c>
     </row>
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>832315</v>
+        <v>832189</v>
       </c>
     </row>
     <row r="3">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>838802</v>
+        <v>838925</v>
       </c>
     </row>
     <row r="5">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>617753</v>
+        <v>617677</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>281200</v>
+        <v>281152</v>
       </c>
     </row>
     <row r="22">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1958799</v>
+        <v>1958793</v>
       </c>
     </row>
     <row r="24">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1057479</v>
+        <v>1057454</v>
       </c>
     </row>
     <row r="30">
@@ -11974,7 +11974,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>114680</v>
+        <v>114675</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
AutomaTivio: comentário sempre bate com a tabela; treemap com nomes e faixas abaixo de 2%
- engine/sincroniza.py: nas frases-padrão do comentário do gestor, cada
  número é trocado pelo valor da tabela (mês, % do benchmark, ano, desde o
  início, CDI+, anualizado, alocação em crédito, carrego, duration). Vale
  para relatório, post e e-mail, porque roda no Contexto.
- Treemap da alocação real: o nome aparece sempre que for legível (duas
  linhas, ou uma linha com corpo menor); itens abaixo de 2% viram faixa no
  pé do último bloco, com nome e valor numa linha.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
+++ b/AutomaTivio/saida/2026-08/conferencia_2026-08.xlsx
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>832189</v>
+        <v>832291</v>
       </c>
     </row>
     <row r="3">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1961063</v>
+        <v>1961067</v>
       </c>
     </row>
     <row r="4">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618536</v>
+        <v>618543</v>
       </c>
     </row>
     <row r="17">
@@ -11734,7 +11734,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>295318</v>
+        <v>295317</v>
       </c>
     </row>
     <row r="18">
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>616870</v>
+        <v>617077</v>
       </c>
     </row>
     <row r="19">
@@ -11764,7 +11764,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>289653</v>
+        <v>289794</v>
       </c>
     </row>
     <row r="20">
@@ -11779,7 +11779,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>617677</v>
+        <v>617709</v>
       </c>
     </row>
     <row r="21">
@@ -11794,7 +11794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>281152</v>
+        <v>281192</v>
       </c>
     </row>
     <row r="22">
@@ -11824,7 +11824,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1958793</v>
+        <v>1958799</v>
       </c>
     </row>
     <row r="24">
@@ -11869,7 +11869,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>833559</v>
+        <v>833617</v>
       </c>
     </row>
     <row r="27">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1959157</v>
+        <v>1959162</v>
       </c>
     </row>
     <row r="28">
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3231558</v>
+        <v>3231856</v>
       </c>
     </row>
     <row r="29">
@@ -11914,7 +11914,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1057454</v>
+        <v>1057746</v>
       </c>
     </row>
     <row r="30">

</xml_diff>